<commit_message>
Remove LaTeX build artifacts; update CV files
Delete generated LaTeX artifacts (cv.log, cv.synctex.gz) and commit updates to cv.tex, cv.pdf and cv.xlsx. A temporary Office lock file (~$cv.xlsx) was accidentally added — consider removing it and adding an ignore rule for such temporary files.
</commit_message>
<xml_diff>
--- a/cv.xlsx
+++ b/cv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzach\Documents\GitHub\cv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62A042B-A341-493E-9A6C-E4F845CE21E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E595E8E6-76CE-4846-BF9C-EFC0D1264E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9060" yWindow="3330" windowWidth="20490" windowHeight="14775" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6030" yWindow="3855" windowWidth="20490" windowHeight="14775" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="work" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="110">
   <si>
     <t>date_start</t>
   </si>
@@ -284,9 +284,6 @@
     <t>Interactive Data Visualization</t>
   </si>
   <si>
-    <t>https://rpubs.com/sedzinfo/covid_deaths_infection</t>
-  </si>
-  <si>
     <t>shiny</t>
   </si>
   <si>
@@ -357,6 +354,12 @@
   </si>
   <si>
     <t>mailto:dzacharatos@yahoo.com</t>
+  </si>
+  <si>
+    <t>grafana</t>
+  </si>
+  <si>
+    <t>https://sedzinfo.grafana.net/public-dashboards/425b920caf1b48dfb15fc829d322e949</t>
   </si>
 </sst>
 </file>
@@ -980,7 +983,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -1013,7 +1016,7 @@
       <c r="C2" t="s">
         <v>46</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1027,7 +1030,7 @@
       <c r="C3" t="s">
         <v>49</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1041,7 +1044,7 @@
       <c r="C4" t="s">
         <v>52</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1055,7 +1058,7 @@
       <c r="C5" t="s">
         <v>55</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1069,7 +1072,7 @@
       <c r="C6" t="s">
         <v>58</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1083,7 +1086,7 @@
       <c r="C7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1097,7 +1100,7 @@
       <c r="C8" t="s">
         <v>64</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1111,7 +1114,7 @@
       <c r="C9" t="s">
         <v>67</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1125,7 +1128,7 @@
       <c r="C10" t="s">
         <v>70</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1139,7 +1142,7 @@
       <c r="C11" t="s">
         <v>73</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1153,7 +1156,7 @@
       <c r="C12" t="s">
         <v>76</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="3" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1167,7 +1170,7 @@
       <c r="C13" t="s">
         <v>80</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="3" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1181,8 +1184,8 @@
       <c r="C14" t="s">
         <v>83</v>
       </c>
-      <c r="D14" t="s">
-        <v>84</v>
+      <c r="D14" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1190,16 +1193,47 @@
         <v>78</v>
       </c>
       <c r="B15" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" t="s">
-        <v>86</v>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{BECD92D5-F8A1-49A5-BFEE-9405B36DF618}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{A386914A-7337-4E29-A64B-73F6E46C3EE2}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{F84F0442-6FCF-4F3E-A2AA-83B9FB2FFD0E}"/>
+    <hyperlink ref="D10" r:id="rId4" xr:uid="{BD614D71-77F1-4C87-990D-F575E3359E29}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{073E7DEE-915D-4A87-A793-99011C509D8C}"/>
+    <hyperlink ref="D15" r:id="rId6" xr:uid="{EC7DD894-97AB-435A-A49B-52D1FD1842C4}"/>
+    <hyperlink ref="D14" r:id="rId7" xr:uid="{2B0C3A3A-CE48-4A22-9390-8D63E794AEE4}"/>
+    <hyperlink ref="D13" r:id="rId8" xr:uid="{D4A5FA8D-3BC1-4641-947A-A07747DAEB45}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{FE43D7FC-D597-410D-95C5-C2FCE8B1C086}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{50B1D3C1-8A33-4F88-B6BB-B490800A4103}"/>
+    <hyperlink ref="D9" r:id="rId11" xr:uid="{A82AF1F4-AB53-4E11-965D-CBA6E5563DE5}"/>
+    <hyperlink ref="D7" r:id="rId12" xr:uid="{C9FED777-0052-42E9-A9DF-7015CE147D66}"/>
+    <hyperlink ref="D4" r:id="rId13" xr:uid="{0B646FE4-7777-4885-855B-400573500F94}"/>
+    <hyperlink ref="D3" r:id="rId14" xr:uid="{DE0801DB-2386-422A-A809-BAAA5F5B0CA7}"/>
+    <hyperlink ref="D16" r:id="rId15" xr:uid="{EDB81896-DB00-45E0-9B5A-FA188C060BA5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1226,41 +1260,41 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" t="s">
         <v>87</v>
-      </c>
-      <c r="B1" t="s">
-        <v>88</v>
       </c>
       <c r="C1" t="s">
         <v>43</v>
       </c>
       <c r="D1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" t="s">
         <v>90</v>
       </c>
-      <c r="B2" t="s">
-        <v>91</v>
-      </c>
       <c r="C2" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" t="s">
         <v>92</v>
       </c>
-      <c r="B3" t="s">
-        <v>93</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D3" s="3">
         <v>6947863817</v>
@@ -1268,58 +1302,58 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" t="s">
         <v>94</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C4" t="s">
-        <v>96</v>
-      </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
         <v>97</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>98</v>
       </c>
-      <c r="C5" t="s">
-        <v>99</v>
-      </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" t="s">
         <v>100</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>101</v>
       </c>
-      <c r="C6" t="s">
-        <v>102</v>
-      </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1327,6 +1361,7 @@
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{EDDDA766-77C7-4001-A642-C6599D449CA2}"/>
     <hyperlink ref="D3" r:id="rId3" display="tel:+306947863817" xr:uid="{231EBA70-480B-46ED-8967-C746082BBB38}"/>
+    <hyperlink ref="C4" r:id="rId4" xr:uid="{F393866C-D4CA-40F7-9BE4-43C1E47FCA89}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1343,12 +1378,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>